<commit_message>
Actualizar agenda y registro
</commit_message>
<xml_diff>
--- a/registro_empates.xlsx
+++ b/registro_empates.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -495,12 +495,45 @@
       <c r="F2" t="n">
         <v>35</v>
       </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
           <t>1520714</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Defensores de Cambaceres vs Berazategui</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Primera C</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="F3" t="n">
+        <v>36.1</v>
+      </c>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>1499945</t>
         </is>
       </c>
     </row>

</xml_diff>